<commit_message>
Update registration and rankings
</commit_message>
<xml_diff>
--- a/Rangliste_Vorlage.xlsx
+++ b/Rangliste_Vorlage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joelz\Dokumente\AeroTrackTiming\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CAC0E60-4F5D-4C1C-8AE1-F2ADC8885F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F10FAE05-DD52-44FE-AB9B-59739AA8A6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24075" yWindow="2430" windowWidth="20820" windowHeight="15285" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rennen 1" sheetId="6" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="14">
   <si>
     <t>Rang</t>
   </si>
@@ -34,9 +34,6 @@
   </si>
   <si>
     <t>Jahrgang</t>
-  </si>
-  <si>
-    <t>Wohnort</t>
   </si>
   <si>
     <t>Rennzeit</t>
@@ -73,7 +70,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -85,6 +82,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -116,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -130,6 +133,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -432,20 +436,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42146104-A206-46E9-B5BB-68F0FBE8D144}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" customWidth="1"/>
     <col min="2" max="3" width="13.28515625" customWidth="1"/>
     <col min="4" max="4" width="10.140625" customWidth="1"/>
-    <col min="5" max="6" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -453,9 +457,8 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -477,11 +480,8 @@
       <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -489,9 +489,8 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -499,11 +498,10 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -511,9 +509,8 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -535,11 +532,8 @@
       <c r="G6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -547,9 +541,8 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -557,11 +550,10 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -569,9 +561,8 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -593,11 +584,8 @@
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -605,9 +593,8 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -615,11 +602,10 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -627,9 +613,8 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>0</v>
       </c>
@@ -651,11 +636,8 @@
       <c r="G14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -663,9 +645,8 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -673,11 +654,10 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -685,9 +665,8 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -709,43 +688,41 @@
       <c r="G18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A17:G17"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.78740157480314965" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;20Rennen 1&amp;RDistanz</oddHeader>
+    <oddFooter>&amp;CAeroTrackTiming</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B318B1E0-113D-4574-8B1C-A809DBF64A6A}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" customWidth="1"/>
     <col min="2" max="3" width="13.28515625" customWidth="1"/>
     <col min="4" max="4" width="10.140625" customWidth="1"/>
-    <col min="5" max="6" width="13.28515625" customWidth="1"/>
-    <col min="7" max="7" width="12.85546875" customWidth="1"/>
-    <col min="8" max="8" width="13.85546875" customWidth="1"/>
+    <col min="5" max="5" width="13.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -753,9 +730,8 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -777,11 +753,8 @@
       <c r="G2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -789,9 +762,8 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -799,11 +771,10 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -811,9 +782,8 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -835,11 +805,8 @@
       <c r="G6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H6" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -847,9 +814,8 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -857,11 +823,10 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -869,9 +834,8 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -893,11 +857,8 @@
       <c r="G10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -905,9 +866,8 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -915,11 +875,10 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -927,9 +886,8 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>0</v>
       </c>
@@ -951,11 +909,8 @@
       <c r="G14" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -963,9 +918,8 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -973,11 +927,10 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -985,9 +938,8 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1009,42 +961,41 @@
       <c r="G18" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H18" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A17:G17"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.78740157480314965" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;20Rennen 2&amp;RDistanz</oddHeader>
+    <oddFooter>&amp;CAeroTrackTiming</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9F5CD02-9D10-4DC1-A5D9-9B12C3774770}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.28515625" customWidth="1"/>
     <col min="2" max="3" width="13.28515625" customWidth="1"/>
     <col min="4" max="4" width="10.140625" customWidth="1"/>
-    <col min="5" max="5" width="13.28515625" customWidth="1"/>
-    <col min="6" max="8" width="12.85546875" customWidth="1"/>
+    <col min="5" max="5" width="12.85546875" customWidth="1"/>
+    <col min="6" max="6" width="20.140625" customWidth="1"/>
+    <col min="7" max="7" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -1052,9 +1003,8 @@
       <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-    </row>
-    <row r="2" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1068,19 +1018,16 @@
         <v>3</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1088,9 +1035,8 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -1098,11 +1044,10 @@
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -1110,9 +1055,8 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
@@ -1126,19 +1070,16 @@
         <v>3</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1146,9 +1087,8 @@
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="C8" s="2"/>
@@ -1156,11 +1096,10 @@
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
@@ -1168,9 +1107,8 @@
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-    </row>
-    <row r="10" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -1184,19 +1122,16 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="C11" s="2"/>
@@ -1204,9 +1139,8 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -1214,11 +1148,10 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -1226,9 +1159,8 @@
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-    </row>
-    <row r="14" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>0</v>
       </c>
@@ -1242,19 +1174,16 @@
         <v>3</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -1262,9 +1191,8 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -1272,11 +1200,10 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
@@ -1284,9 +1211,8 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:7" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1300,31 +1226,32 @@
         <v>3</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>13</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="6:6" x14ac:dyDescent="0.25">
+      <c r="F47" s="5"/>
+    </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A17:G17"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.78740157480314965" bottom="0.51181102362204722" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;20Gesamtwertung</oddHeader>
+    <oddFooter>&amp;CAeroTrackTiming</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>